<commit_message>
Analysis for task 2_6 data
</commit_message>
<xml_diff>
--- a/data/electrical/task_2_6.xlsx
+++ b/data/electrical/task_2_6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/sd3525_ic_ac_uk/Documents/waves/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\GitHub\laboratory-waves\data\electrical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="580" documentId="8_{67420F97-00E5-49CE-B2EF-DDD35DE2EC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB3D8B0F-E14B-4557-A1D0-DD888EDE4DE7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D4D5CE-6880-43FC-8C8B-8E5617F47709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D73005F2-5D69-4685-BA2C-A4D36748CC2D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D73005F2-5D69-4685-BA2C-A4D36748CC2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -91,10 +91,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.0000000"/>
-    <numFmt numFmtId="173" formatCode="0.000E+00"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000000"/>
+    <numFmt numFmtId="167" formatCode="0.000E+00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -131,9 +131,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -141,16 +141,15 @@
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -169,7 +168,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -684,7 +683,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -983,7 +981,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1888,7 +1886,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4559,12 +4557,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -4881,54 +4875,54 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1926CA6-FD9C-49C3-B77C-956FA8CD82CE}">
   <dimension ref="A1:O48"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="7" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" customWidth="1"/>
-    <col min="7" max="8" width="10.28515625" customWidth="1"/>
-    <col min="12" max="13" width="19.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" customWidth="1"/>
-    <col min="16" max="16" width="10.28515625" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="8" width="10.33203125" customWidth="1"/>
+    <col min="12" max="13" width="19.44140625" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" customWidth="1"/>
+    <col min="16" max="16" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B1">
         <v>38</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>9</v>
       </c>
       <c r="D1">
         <v>5</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F1">
         <v>143069.65</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F2" t="s">
@@ -4959,40 +4953,40 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>0</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="3">
-        <v>33</v>
-      </c>
-      <c r="D3" s="6">
-        <f>PI()*A3/$B$1</f>
+      <c r="C3">
         <v>0</v>
       </c>
-      <c r="E3" s="7">
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D18" si="0">PI()*A3/$B$1</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="6">
         <v>20</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>2.1320000000000001</v>
       </c>
       <c r="G3">
         <v>1E-3</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>1.89</v>
       </c>
       <c r="I3">
         <v>0.01</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="4">
         <f>H3/F3</f>
         <v>0.88649155722326445</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="4">
         <f>SQRT((I3/F3)^2+(G3*H3/F3^2)^2)</f>
         <v>4.7088257352182481E-3</v>
       </c>
@@ -5009,1657 +5003,1644 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" s="6">
-        <f>PI()*A4/$B$1</f>
+      <c r="D4" s="5">
+        <f t="shared" si="0"/>
         <v>8.2673490883941922E-2</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>5900</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>2.5499999999999998</v>
       </c>
       <c r="G4">
         <v>0.01</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>2.34</v>
       </c>
       <c r="I4">
         <v>0.01</v>
       </c>
-      <c r="J4" s="5">
-        <f t="shared" ref="J4:J35" si="0">H4/F4</f>
+      <c r="J4" s="4">
+        <f t="shared" ref="J4:J35" si="1">H4/F4</f>
         <v>0.91764705882352937</v>
       </c>
-      <c r="K4" s="5">
-        <f t="shared" ref="K4:K23" si="1">SQRT((I4/F4)^2+(G4*H4/F4^2)^2)</f>
+      <c r="K4" s="4">
+        <f t="shared" ref="K4:K23" si="2">SQRT((I4/F4)^2+(G4*H4/F4^2)^2)</f>
         <v>5.3224747080253716E-3</v>
       </c>
-      <c r="L4" s="9">
-        <f t="shared" ref="L4:L35" si="2">E4*2*PI()/D4</f>
+      <c r="L4" s="8">
+        <f t="shared" ref="L4:L35" si="3">E4*2*PI()/D4</f>
         <v>448400</v>
       </c>
-      <c r="M4" s="8">
-        <f>(E4-E3)*2*PI()/(D4-D3)</f>
+      <c r="M4" s="7">
+        <f t="shared" ref="M4:M35" si="4">(E4-E3)*2*PI()/(D4-D3)</f>
         <v>446880</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N35" si="3">$F$1*SIN(D4/2)</f>
+        <f t="shared" ref="N4:N35" si="5">$F$1*SIN(D4/2)</f>
         <v>5912.3496020367184</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>2</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="6">
-        <f>PI()*A5/$B$1</f>
+      <c r="D5" s="5">
+        <f t="shared" si="0"/>
         <v>0.16534698176788384</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>11800</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>2.4</v>
       </c>
       <c r="G5">
         <v>0.01</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <v>2.2799999999999998</v>
       </c>
       <c r="I5">
         <v>0.01</v>
       </c>
-      <c r="J5" s="5">
-        <f t="shared" si="0"/>
+      <c r="J5" s="4">
+        <f t="shared" si="1"/>
         <v>0.95</v>
       </c>
-      <c r="K5" s="5">
-        <f t="shared" si="1"/>
+      <c r="K5" s="4">
+        <f t="shared" si="2"/>
         <v>5.7471309267223833E-3</v>
       </c>
-      <c r="L5" s="9">
-        <f t="shared" si="2"/>
+      <c r="L5" s="8">
+        <f t="shared" si="3"/>
         <v>448400</v>
       </c>
-      <c r="M5" s="8">
-        <f>(E5-E4)*2*PI()/(D5-D4)</f>
+      <c r="M5" s="7">
+        <f t="shared" si="4"/>
         <v>448400</v>
       </c>
       <c r="N5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>11814.598053955669</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>3</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6" s="3">
-        <v>5</v>
-      </c>
-      <c r="D6" s="6">
-        <f>PI()*A6/$B$1</f>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="0"/>
         <v>0.24802047265182578</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>17800</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>2.4500000000000002</v>
       </c>
       <c r="G6">
         <v>0.01</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>2.2200000000000002</v>
       </c>
       <c r="I6">
         <v>0.01</v>
       </c>
-      <c r="J6" s="5">
-        <f t="shared" si="0"/>
+      <c r="J6" s="4">
+        <f t="shared" si="1"/>
         <v>0.90612244897959182</v>
       </c>
-      <c r="K6" s="5">
-        <f t="shared" si="1"/>
+      <c r="K6" s="4">
+        <f t="shared" si="2"/>
         <v>5.5080235935815883E-3</v>
       </c>
-      <c r="L6" s="9">
-        <f t="shared" si="2"/>
+      <c r="L6" s="8">
+        <f t="shared" si="3"/>
         <v>450933.33333333331</v>
       </c>
-      <c r="M6" s="8">
-        <f>(E6-E5)*2*PI()/(D6-D5)</f>
+      <c r="M6" s="7">
+        <f t="shared" si="4"/>
         <v>455999.99999999994</v>
       </c>
       <c r="N6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>17696.661463284618</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>4</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" s="3">
-        <v>6</v>
-      </c>
-      <c r="D7" s="6">
-        <f>PI()*A7/$B$1</f>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="0"/>
         <v>0.33069396353576769</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>23600</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>2.66</v>
       </c>
       <c r="G7">
         <v>0.01</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="3">
         <v>2.17</v>
       </c>
       <c r="I7">
         <v>0.01</v>
       </c>
-      <c r="J7" s="5">
-        <f t="shared" si="0"/>
+      <c r="J7" s="4">
+        <f t="shared" si="1"/>
         <v>0.81578947368421051</v>
       </c>
-      <c r="K7" s="5">
-        <f t="shared" si="1"/>
+      <c r="K7" s="4">
+        <f t="shared" si="2"/>
         <v>4.8516817709692234E-3</v>
       </c>
-      <c r="L7" s="9">
-        <f t="shared" si="2"/>
+      <c r="L7" s="8">
+        <f t="shared" si="3"/>
         <v>448400</v>
       </c>
-      <c r="M7" s="8">
-        <f>(E7-E6)*2*PI()/(D7-D6)</f>
+      <c r="M7" s="7">
+        <f t="shared" si="4"/>
         <v>440800.00000000006</v>
       </c>
       <c r="N7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>23548.490423357998</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>5</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
-      <c r="C8" s="3">
-        <v>3</v>
-      </c>
-      <c r="D8" s="6">
-        <f>PI()*A8/$B$1</f>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="0"/>
         <v>0.41336745441970962</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>29500</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>2.46</v>
       </c>
       <c r="G8">
         <v>0.01</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>2.1</v>
       </c>
       <c r="I8">
         <v>0.01</v>
       </c>
-      <c r="J8" s="5">
-        <f t="shared" si="0"/>
+      <c r="J8" s="4">
+        <f t="shared" si="1"/>
         <v>0.85365853658536595</v>
       </c>
-      <c r="K8" s="5">
-        <f t="shared" si="1"/>
+      <c r="K8" s="4">
+        <f t="shared" si="2"/>
         <v>5.344767785819376E-3</v>
       </c>
-      <c r="L8" s="9">
-        <f t="shared" si="2"/>
+      <c r="L8" s="8">
+        <f t="shared" si="3"/>
         <v>448400</v>
       </c>
-      <c r="M8" s="8">
-        <f>(E8-E7)*2*PI()/(D8-D7)</f>
+      <c r="M8" s="7">
+        <f t="shared" si="4"/>
         <v>448399.99999999994</v>
       </c>
       <c r="N8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>29360.087182559626</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>6</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
-      <c r="C9" s="3">
-        <v>4</v>
-      </c>
-      <c r="D9" s="6">
-        <f>PI()*A9/$B$1</f>
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" si="0"/>
         <v>0.49604094530365156</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <v>35200</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>2.52</v>
       </c>
       <c r="G9">
         <v>0.01</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>2</v>
       </c>
       <c r="I9">
         <v>0.01</v>
       </c>
-      <c r="J9" s="5">
-        <f t="shared" si="0"/>
+      <c r="J9" s="4">
+        <f t="shared" si="1"/>
         <v>0.79365079365079361</v>
       </c>
-      <c r="K9" s="5">
-        <f t="shared" si="1"/>
+      <c r="K9" s="4">
+        <f t="shared" si="2"/>
         <v>5.0661434788606434E-3</v>
       </c>
-      <c r="L9" s="9">
-        <f t="shared" si="2"/>
+      <c r="L9" s="8">
+        <f t="shared" si="3"/>
         <v>445866.66666666669</v>
       </c>
-      <c r="M9" s="8">
-        <f>(E9-E8)*2*PI()/(D9-D8)</f>
+      <c r="M9" s="7">
+        <f t="shared" si="4"/>
         <v>433199.99999999988</v>
       </c>
       <c r="N9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>35121.522725313633</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>7</v>
       </c>
       <c r="B10">
         <v>0</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10">
         <v>7</v>
       </c>
-      <c r="D10" s="6">
-        <f>PI()*A10/$B$1</f>
+      <c r="D10" s="5">
+        <f t="shared" si="0"/>
         <v>0.57871443618759344</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <v>41200</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>2.5</v>
       </c>
       <c r="G10">
         <v>0.01</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>1.95</v>
       </c>
       <c r="I10">
         <v>0.01</v>
       </c>
-      <c r="J10" s="5">
-        <f t="shared" si="0"/>
+      <c r="J10" s="4">
+        <f t="shared" si="1"/>
         <v>0.78</v>
       </c>
-      <c r="K10" s="5">
-        <f t="shared" si="1"/>
+      <c r="K10" s="4">
+        <f t="shared" si="2"/>
         <v>5.0729084359960605E-3</v>
       </c>
-      <c r="L10" s="9">
-        <f t="shared" si="2"/>
+      <c r="L10" s="8">
+        <f t="shared" si="3"/>
         <v>447314.28571428574</v>
       </c>
-      <c r="M10" s="8">
-        <f>(E10-E9)*2*PI()/(D10-D9)</f>
+      <c r="M10" s="7">
+        <f t="shared" si="4"/>
         <v>456000.00000000023</v>
       </c>
       <c r="N10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>40822.953735641</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>8</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11">
         <v>8</v>
       </c>
-      <c r="D11" s="6">
-        <f>PI()*A11/$B$1</f>
+      <c r="D11" s="5">
+        <f t="shared" si="0"/>
         <v>0.66138792707153538</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <v>46700</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>2.29</v>
       </c>
       <c r="G11">
         <v>0.01</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>1.89</v>
       </c>
       <c r="I11">
         <v>0.01</v>
       </c>
-      <c r="J11" s="5">
-        <f t="shared" si="0"/>
+      <c r="J11" s="4">
+        <f t="shared" si="1"/>
         <v>0.82532751091703049</v>
       </c>
-      <c r="K11" s="5">
-        <f t="shared" si="1"/>
+      <c r="K11" s="4">
+        <f t="shared" si="2"/>
         <v>5.6619985293600269E-3</v>
       </c>
-      <c r="L11" s="9">
-        <f t="shared" si="2"/>
+      <c r="L11" s="8">
+        <f t="shared" si="3"/>
         <v>443650</v>
       </c>
-      <c r="M11" s="8">
-        <f>(E11-E10)*2*PI()/(D11-D10)</f>
+      <c r="M11" s="7">
+        <f t="shared" si="4"/>
         <v>417999.99999999988</v>
       </c>
       <c r="N11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>46454.63941429984</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>9</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12">
         <v>0</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12">
         <v>9</v>
       </c>
-      <c r="D12" s="6">
-        <f>PI()*A12/$B$1</f>
+      <c r="D12" s="5">
+        <f t="shared" si="0"/>
         <v>0.74406141795547731</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <v>52200</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>2.5299999999999998</v>
       </c>
       <c r="G12">
         <v>0.01</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>1.83</v>
       </c>
       <c r="I12">
         <v>0.01</v>
       </c>
-      <c r="J12" s="5">
-        <f t="shared" si="0"/>
+      <c r="J12" s="4">
+        <f t="shared" si="1"/>
         <v>0.72332015810276684</v>
       </c>
-      <c r="K12" s="5">
-        <f t="shared" si="1"/>
+      <c r="K12" s="4">
+        <f t="shared" si="2"/>
         <v>4.8781686534771721E-3</v>
       </c>
-      <c r="L12" s="9">
-        <f t="shared" si="2"/>
+      <c r="L12" s="8">
+        <f t="shared" si="3"/>
         <v>440800</v>
       </c>
-      <c r="M12" s="8">
-        <f>(E12-E11)*2*PI()/(D12-D11)</f>
+      <c r="M12" s="7">
+        <f t="shared" si="4"/>
         <v>417999.99999999988</v>
       </c>
       <c r="N12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>52006.958120777432</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>10</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13">
         <v>1</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13">
         <v>10</v>
       </c>
-      <c r="D13" s="6">
-        <f>PI()*A13/$B$1</f>
+      <c r="D13" s="5">
+        <f t="shared" si="0"/>
         <v>0.82673490883941925</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <v>57700</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>2.6</v>
       </c>
       <c r="G13">
         <v>0.01</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>1.76</v>
       </c>
       <c r="I13">
         <v>0.01</v>
       </c>
-      <c r="J13" s="5">
-        <f t="shared" si="0"/>
+      <c r="J13" s="4">
+        <f t="shared" si="1"/>
         <v>0.67692307692307685</v>
       </c>
-      <c r="K13" s="5">
-        <f t="shared" si="1"/>
+      <c r="K13" s="4">
+        <f t="shared" si="2"/>
         <v>4.6444992788616342E-3</v>
       </c>
-      <c r="L13" s="9">
-        <f t="shared" si="2"/>
+      <c r="L13" s="8">
+        <f t="shared" si="3"/>
         <v>438520</v>
       </c>
-      <c r="M13" s="8">
-        <f>(E13-E12)*2*PI()/(D13-D12)</f>
+      <c r="M13" s="7">
+        <f t="shared" si="4"/>
         <v>417999.99999999988</v>
       </c>
       <c r="N13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>57470.423811701701</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>11</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14">
         <v>0</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14">
         <v>11</v>
       </c>
-      <c r="D14" s="6">
-        <f>PI()*A14/$B$1</f>
+      <c r="D14" s="5">
+        <f t="shared" si="0"/>
         <v>0.90940839972336107</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="6">
         <v>63500</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>2.98</v>
       </c>
       <c r="G14">
         <v>0.01</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>1.67</v>
       </c>
       <c r="I14">
         <v>0.01</v>
       </c>
-      <c r="J14" s="5">
-        <f t="shared" si="0"/>
+      <c r="J14" s="4">
+        <f t="shared" si="1"/>
         <v>0.56040268456375841</v>
       </c>
-      <c r="K14" s="5">
-        <f t="shared" si="1"/>
+      <c r="K14" s="4">
+        <f t="shared" si="2"/>
         <v>3.846713790030877E-3</v>
       </c>
-      <c r="L14" s="9">
-        <f t="shared" si="2"/>
+      <c r="L14" s="8">
+        <f t="shared" si="3"/>
         <v>438727.27272727276</v>
       </c>
-      <c r="M14" s="8">
-        <f>(E14-E13)*2*PI()/(D14-D13)</f>
+      <c r="M14" s="7">
+        <f t="shared" si="4"/>
         <v>440800.00000000052</v>
       </c>
       <c r="N14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>62835.702247587171</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>12</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15">
         <v>1</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15">
         <v>12</v>
       </c>
-      <c r="D15" s="6">
-        <f>PI()*A15/$B$1</f>
+      <c r="D15" s="5">
+        <f t="shared" si="0"/>
         <v>0.99208189060730312</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <v>69300</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>2.2799999999999998</v>
       </c>
       <c r="G15">
         <v>0.01</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="3">
         <v>1.47</v>
       </c>
       <c r="I15">
         <v>0.01</v>
       </c>
-      <c r="J15" s="5">
-        <f t="shared" si="0"/>
+      <c r="J15" s="4">
+        <f t="shared" si="1"/>
         <v>0.64473684210526316</v>
       </c>
-      <c r="K15" s="5">
-        <f t="shared" si="1"/>
+      <c r="K15" s="4">
+        <f t="shared" si="2"/>
         <v>5.2185345076769625E-3</v>
       </c>
-      <c r="L15" s="9">
-        <f t="shared" si="2"/>
+      <c r="L15" s="8">
+        <f t="shared" si="3"/>
         <v>438900</v>
       </c>
-      <c r="M15" s="8">
-        <f>(E15-E14)*2*PI()/(D15-D14)</f>
+      <c r="M15" s="7">
+        <f t="shared" si="4"/>
         <v>440799.9999999993</v>
       </c>
       <c r="N15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>68093.626940226546</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>13</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16">
         <v>0</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16">
         <v>13</v>
       </c>
-      <c r="D16" s="6">
-        <f>PI()*A16/$B$1</f>
+      <c r="D16" s="5">
+        <f t="shared" si="0"/>
         <v>1.0747553814912452</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="6">
         <v>73800</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>2.91</v>
       </c>
       <c r="G16">
         <v>0.01</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="3">
         <v>1.43</v>
       </c>
       <c r="I16">
         <v>0.01</v>
       </c>
-      <c r="J16" s="5">
-        <f t="shared" si="0"/>
+      <c r="J16" s="4">
+        <f t="shared" si="1"/>
         <v>0.49140893470790376</v>
       </c>
-      <c r="K16" s="5">
-        <f t="shared" si="1"/>
+      <c r="K16" s="4">
+        <f t="shared" si="2"/>
         <v>3.8289293610729793E-3</v>
       </c>
-      <c r="L16" s="9">
-        <f t="shared" si="2"/>
+      <c r="L16" s="8">
+        <f t="shared" si="3"/>
         <v>431446.15384615381</v>
       </c>
-      <c r="M16" s="8">
-        <f>(E16-E15)*2*PI()/(D16-D15)</f>
+      <c r="M16" s="7">
+        <f t="shared" si="4"/>
         <v>341999.99999999953</v>
       </c>
       <c r="N16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>73235.214813482045</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>14</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17">
         <v>1</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17">
         <v>14</v>
       </c>
-      <c r="D17" s="6">
-        <f>PI()*A17/$B$1</f>
+      <c r="D17" s="5">
+        <f t="shared" si="0"/>
         <v>1.1574288723751869</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="6">
         <v>79500</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>2.7</v>
       </c>
       <c r="G17">
         <v>0.01</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="3">
         <v>1.49</v>
       </c>
       <c r="I17">
         <v>0.01</v>
       </c>
-      <c r="J17" s="5">
-        <f t="shared" si="0"/>
+      <c r="J17" s="4">
+        <f t="shared" si="1"/>
         <v>0.55185185185185182</v>
       </c>
-      <c r="K17" s="5">
-        <f t="shared" si="1"/>
+      <c r="K17" s="4">
+        <f t="shared" si="2"/>
         <v>4.2302400584226484E-3</v>
       </c>
-      <c r="L17" s="9">
-        <f t="shared" si="2"/>
+      <c r="L17" s="8">
+        <f t="shared" si="3"/>
         <v>431571.42857142858</v>
       </c>
-      <c r="M17" s="8">
-        <f>(E17-E16)*2*PI()/(D17-D16)</f>
+      <c r="M17" s="7">
+        <f t="shared" si="4"/>
         <v>433200.00000000105</v>
       </c>
       <c r="N17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>78251.681550720255</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>15</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18">
         <v>0</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18">
         <v>15</v>
       </c>
-      <c r="D18" s="6">
-        <f>PI()*A18/$B$1</f>
+      <c r="D18" s="5">
+        <f t="shared" si="0"/>
         <v>1.2401023632591288</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="6">
         <v>84000</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>2.65</v>
       </c>
       <c r="G18">
         <v>0.01</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>1.4</v>
       </c>
       <c r="I18">
         <v>0.01</v>
       </c>
-      <c r="J18" s="5">
-        <f t="shared" si="0"/>
+      <c r="J18" s="4">
+        <f t="shared" si="1"/>
         <v>0.52830188679245282</v>
       </c>
-      <c r="K18" s="5">
-        <f t="shared" si="1"/>
+      <c r="K18" s="4">
+        <f t="shared" si="2"/>
         <v>4.2678275744095998E-3</v>
       </c>
-      <c r="L18" s="9">
-        <f t="shared" si="2"/>
+      <c r="L18" s="8">
+        <f t="shared" si="3"/>
         <v>425600</v>
       </c>
-      <c r="M18" s="8">
-        <f>(E18-E17)*2*PI()/(D18-D17)</f>
+      <c r="M18" s="7">
+        <f t="shared" si="4"/>
         <v>341999.99999999994</v>
       </c>
       <c r="N18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>83134.456602669903</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>16</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19">
         <v>1</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19">
         <v>16</v>
       </c>
-      <c r="D19" s="6">
-        <f t="shared" ref="D19:D35" si="4">PI()*A19/$B$1</f>
+      <c r="D19" s="5">
+        <f t="shared" ref="D19:D35" si="6">PI()*A19/$B$1</f>
         <v>1.3227758541430708</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="6">
         <v>89200</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>3.22</v>
       </c>
       <c r="G19">
         <v>0.01</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>1.27</v>
       </c>
       <c r="I19">
         <v>0.01</v>
       </c>
-      <c r="J19" s="5">
-        <f t="shared" si="0"/>
+      <c r="J19" s="4">
+        <f t="shared" si="1"/>
         <v>0.39440993788819873</v>
       </c>
-      <c r="K19" s="5">
-        <f t="shared" si="1"/>
+      <c r="K19" s="4">
+        <f t="shared" si="2"/>
         <v>3.3384142686238277E-3</v>
       </c>
-      <c r="L19" s="9">
-        <f t="shared" si="2"/>
+      <c r="L19" s="8">
+        <f t="shared" si="3"/>
         <v>423700</v>
       </c>
-      <c r="M19" s="8">
-        <f>(E19-E18)*2*PI()/(D19-D18)</f>
+      <c r="M19" s="7">
+        <f t="shared" si="4"/>
         <v>395199.99999999994</v>
       </c>
       <c r="N19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>87875.197830061326</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>17</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20">
         <v>0</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20">
         <v>17</v>
       </c>
-      <c r="D20" s="6">
-        <f t="shared" si="4"/>
+      <c r="D20" s="5">
+        <f t="shared" si="6"/>
         <v>1.4054493450270129</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6">
         <v>93850</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>2.0099999999999998</v>
       </c>
       <c r="G20">
         <v>0.01</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="3">
         <v>1.2</v>
       </c>
       <c r="I20">
         <v>0.01</v>
       </c>
-      <c r="J20" s="5">
-        <f t="shared" si="0"/>
+      <c r="J20" s="4">
+        <f t="shared" si="1"/>
         <v>0.59701492537313439</v>
       </c>
-      <c r="K20" s="5">
-        <f t="shared" si="1"/>
+      <c r="K20" s="4">
+        <f t="shared" si="2"/>
         <v>5.7943153411745473E-3</v>
       </c>
-      <c r="L20" s="9">
-        <f t="shared" si="2"/>
+      <c r="L20" s="8">
+        <f t="shared" si="3"/>
         <v>419564.70588235289</v>
       </c>
-      <c r="M20" s="8">
-        <f>(E20-E19)*2*PI()/(D20-D19)</f>
+      <c r="M20" s="7">
+        <f t="shared" si="4"/>
         <v>353399.99999999901</v>
       </c>
       <c r="N20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>92465.805756031565</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>18</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21">
         <v>1</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21">
         <v>18</v>
       </c>
-      <c r="D21" s="6">
-        <f t="shared" si="4"/>
+      <c r="D21" s="5">
+        <f t="shared" si="6"/>
         <v>1.4881228359109546</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="6">
         <v>98300</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="3">
         <v>3.15</v>
       </c>
       <c r="G21">
         <v>0.01</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="3">
         <v>1.1100000000000001</v>
       </c>
       <c r="I21">
         <v>0.01</v>
       </c>
-      <c r="J21" s="5">
-        <f t="shared" si="0"/>
+      <c r="J21" s="4">
+        <f t="shared" si="1"/>
         <v>0.35238095238095241</v>
       </c>
-      <c r="K21" s="5">
-        <f t="shared" si="1"/>
+      <c r="K21" s="4">
+        <f t="shared" si="2"/>
         <v>3.3659363023897373E-3</v>
       </c>
-      <c r="L21" s="9">
-        <f t="shared" si="2"/>
+      <c r="L21" s="8">
+        <f t="shared" si="3"/>
         <v>415044.4444444445</v>
       </c>
-      <c r="M21" s="8">
-        <f>(E21-E20)*2*PI()/(D21-D20)</f>
+      <c r="M21" s="7">
+        <f t="shared" si="4"/>
         <v>338200.00000000087</v>
       </c>
       <c r="N21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>96898.437403944699</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>19</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22">
         <v>0</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22">
         <v>19</v>
       </c>
-      <c r="D22" s="6">
-        <f t="shared" si="4"/>
+      <c r="D22" s="5">
+        <f t="shared" si="6"/>
         <v>1.5707963267948966</v>
       </c>
-      <c r="E22" s="7">
+      <c r="E22" s="6">
         <v>102400</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="3">
         <v>2.68</v>
       </c>
       <c r="G22">
         <v>0.01</v>
       </c>
-      <c r="H22" s="4">
+      <c r="H22" s="3">
         <v>0.87</v>
       </c>
       <c r="I22">
         <v>0.01</v>
       </c>
-      <c r="J22" s="5">
-        <f t="shared" si="0"/>
+      <c r="J22" s="4">
+        <f t="shared" si="1"/>
         <v>0.32462686567164178</v>
       </c>
-      <c r="K22" s="5">
-        <f t="shared" si="1"/>
+      <c r="K22" s="4">
+        <f t="shared" si="2"/>
         <v>3.9230289981498478E-3</v>
       </c>
-      <c r="L22" s="9">
-        <f t="shared" si="2"/>
+      <c r="L22" s="8">
+        <f t="shared" si="3"/>
         <v>409600</v>
       </c>
-      <c r="M22" s="8">
-        <f>(E22-E21)*2*PI()/(D22-D21)</f>
+      <c r="M22" s="7">
+        <f t="shared" si="4"/>
         <v>311599.99999999994</v>
       </c>
       <c r="N22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>101165.51969698592</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>20</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23">
         <v>20</v>
       </c>
-      <c r="D23" s="6">
-        <f t="shared" si="4"/>
+      <c r="D23" s="5">
+        <f t="shared" si="6"/>
         <v>1.6534698176788385</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="6">
         <v>107750</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="3">
         <v>3.61</v>
       </c>
       <c r="G23">
         <v>0.01</v>
       </c>
-      <c r="H23" s="4">
+      <c r="H23" s="3">
         <v>0.97</v>
       </c>
       <c r="I23">
         <v>0.01</v>
       </c>
-      <c r="J23" s="5">
-        <f t="shared" si="0"/>
+      <c r="J23" s="4">
+        <f t="shared" si="1"/>
         <v>0.26869806094182824</v>
       </c>
-      <c r="K23" s="5">
-        <f t="shared" si="1"/>
+      <c r="K23" s="4">
+        <f t="shared" si="2"/>
         <v>2.8683386551241236E-3</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="8">
         <f>E23*2*PI()/D23</f>
         <v>409450</v>
       </c>
-      <c r="M23" s="8">
-        <f>(E23-E22)*2*PI()/(D23-D22)</f>
+      <c r="M23" s="7">
+        <f t="shared" si="4"/>
         <v>406599.99999999994</v>
       </c>
       <c r="N23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>105259.7623966362</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>21</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24">
         <v>0</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24">
         <v>21</v>
       </c>
-      <c r="D24" s="6">
-        <f t="shared" si="4"/>
+      <c r="D24" s="5">
+        <f t="shared" si="6"/>
         <v>1.7361433085627804</v>
       </c>
-      <c r="E24" s="7">
+      <c r="E24" s="6">
         <v>111500</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="3">
         <v>3.19</v>
       </c>
       <c r="G24">
         <v>0.01</v>
       </c>
-      <c r="H24" s="4">
+      <c r="H24" s="3">
         <v>0.91</v>
       </c>
       <c r="I24">
         <v>0.01</v>
       </c>
-      <c r="J24" s="5">
-        <f t="shared" si="0"/>
+      <c r="J24" s="4">
+        <f t="shared" si="1"/>
         <v>0.28526645768025077</v>
       </c>
-      <c r="K24" s="5">
-        <f t="shared" ref="K4:K35" si="5">I24/F24+G24*H24/F24^2</f>
+      <c r="K24" s="4">
+        <f t="shared" ref="K24:K35" si="7">I24/F24+G24*H24/F24^2</f>
         <v>4.0290484566779024E-3</v>
       </c>
-      <c r="L24" s="9">
-        <f t="shared" si="2"/>
+      <c r="L24" s="8">
+        <f t="shared" si="3"/>
         <v>403523.80952380953</v>
       </c>
-      <c r="M24" s="8">
-        <f>(E24-E23)*2*PI()/(D24-D23)</f>
+      <c r="M24" s="7">
+        <f t="shared" si="4"/>
         <v>284999.99999999994</v>
       </c>
       <c r="N24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>109174.17055792244</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>22</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25">
         <v>1</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C25">
         <v>22</v>
       </c>
-      <c r="D25" s="6">
-        <f t="shared" si="4"/>
+      <c r="D25" s="5">
+        <f t="shared" si="6"/>
         <v>1.8188167994467221</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
         <v>116100</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="3">
         <v>2.72</v>
       </c>
       <c r="G25">
         <v>0.01</v>
       </c>
-      <c r="H25" s="4">
+      <c r="H25" s="3">
         <v>0.82</v>
       </c>
       <c r="I25">
         <v>0.01</v>
       </c>
-      <c r="J25" s="5">
-        <f t="shared" si="0"/>
+      <c r="J25" s="4">
+        <f t="shared" si="1"/>
         <v>0.3014705882352941</v>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="4">
+        <f t="shared" si="7"/>
+        <v>4.7848183391003456E-3</v>
+      </c>
+      <c r="L25" s="8">
+        <f t="shared" si="3"/>
+        <v>401072.72727272729</v>
+      </c>
+      <c r="M25" s="7">
+        <f t="shared" si="4"/>
+        <v>349600.00000000087</v>
+      </c>
+      <c r="N25">
         <f t="shared" si="5"/>
-        <v>4.7848183391003456E-3</v>
-      </c>
-      <c r="L25" s="9">
-        <f t="shared" si="2"/>
-        <v>401072.72727272729</v>
-      </c>
-      <c r="M25" s="8">
-        <f>(E25-E24)*2*PI()/(D25-D24)</f>
-        <v>349600.00000000087</v>
-      </c>
-      <c r="N25">
-        <f t="shared" si="3"/>
         <v>112902.05648016374</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>23</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26">
         <v>0</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26">
         <v>23</v>
       </c>
-      <c r="D26" s="6">
-        <f t="shared" si="4"/>
+      <c r="D26" s="5">
+        <f t="shared" si="6"/>
         <v>1.9014902903306641</v>
       </c>
-      <c r="E26" s="7">
+      <c r="E26" s="6">
         <v>119200</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="3">
         <v>2.85</v>
       </c>
       <c r="G26">
         <v>0.01</v>
       </c>
-      <c r="H26" s="4">
+      <c r="H26" s="3">
         <v>0.78</v>
       </c>
       <c r="I26">
         <v>0.01</v>
       </c>
-      <c r="J26" s="5">
-        <f t="shared" si="0"/>
+      <c r="J26" s="4">
+        <f t="shared" si="1"/>
         <v>0.27368421052631581</v>
       </c>
-      <c r="K26" s="5">
+      <c r="K26" s="4">
+        <f t="shared" si="7"/>
+        <v>4.4690674053554941E-3</v>
+      </c>
+      <c r="L26" s="8">
+        <f t="shared" si="3"/>
+        <v>393878.26086956525</v>
+      </c>
+      <c r="M26" s="7">
+        <f t="shared" si="4"/>
+        <v>235599.99999999997</v>
+      </c>
+      <c r="N26">
         <f t="shared" si="5"/>
-        <v>4.4690674053554941E-3</v>
-      </c>
-      <c r="L26" s="9">
-        <f t="shared" si="2"/>
-        <v>393878.26086956525</v>
-      </c>
-      <c r="M26" s="8">
-        <f>(E26-E25)*2*PI()/(D26-D25)</f>
-        <v>235599.99999999997</v>
-      </c>
-      <c r="N26">
-        <f t="shared" si="3"/>
         <v>116437.05113279574</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>24</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B27">
         <v>1</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C27">
         <v>24</v>
       </c>
-      <c r="D27" s="6">
-        <f t="shared" si="4"/>
+      <c r="D27" s="5">
+        <f t="shared" si="6"/>
         <v>1.9841637812146062</v>
       </c>
-      <c r="E27" s="7">
+      <c r="E27" s="6">
         <v>123000</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="3">
         <v>3.18</v>
       </c>
       <c r="G27">
         <v>0.01</v>
       </c>
-      <c r="H27" s="4">
+      <c r="H27" s="3">
         <v>0.72</v>
       </c>
       <c r="I27">
         <v>0.01</v>
       </c>
-      <c r="J27" s="5">
-        <f t="shared" si="0"/>
+      <c r="J27" s="4">
+        <f t="shared" si="1"/>
         <v>0.22641509433962262</v>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="4">
+        <f t="shared" si="7"/>
+        <v>3.8566512400617062E-3</v>
+      </c>
+      <c r="L27" s="8">
+        <f t="shared" si="3"/>
+        <v>389500</v>
+      </c>
+      <c r="M27" s="7">
+        <f t="shared" si="4"/>
+        <v>288799.99999999919</v>
+      </c>
+      <c r="N27">
         <f t="shared" si="5"/>
-        <v>3.8566512400617062E-3</v>
-      </c>
-      <c r="L27" s="9">
-        <f t="shared" si="2"/>
-        <v>389500</v>
-      </c>
-      <c r="M27" s="8">
-        <f>(E27-E26)*2*PI()/(D27-D26)</f>
-        <v>288799.99999999919</v>
-      </c>
-      <c r="N27">
-        <f t="shared" si="3"/>
         <v>119773.11503675256</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>25</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28">
         <v>0</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28">
         <v>25</v>
       </c>
-      <c r="D28" s="6">
-        <f t="shared" si="4"/>
+      <c r="D28" s="5">
+        <f t="shared" si="6"/>
         <v>2.0668372720985482</v>
       </c>
-      <c r="E28" s="7">
+      <c r="E28" s="6">
         <v>126100</v>
       </c>
-      <c r="F28" s="4">
+      <c r="F28" s="3">
         <v>2.89</v>
       </c>
       <c r="G28">
         <v>0.01</v>
       </c>
-      <c r="H28" s="4">
+      <c r="H28" s="3">
         <v>0.56999999999999995</v>
       </c>
       <c r="I28">
         <v>0.01</v>
       </c>
-      <c r="J28" s="5">
-        <f t="shared" si="0"/>
+      <c r="J28" s="4">
+        <f t="shared" si="1"/>
         <v>0.19723183391003457</v>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="4">
+        <f t="shared" si="7"/>
+        <v>4.142670705571054E-3</v>
+      </c>
+      <c r="L28" s="8">
+        <f t="shared" si="3"/>
+        <v>383344</v>
+      </c>
+      <c r="M28" s="7">
+        <f t="shared" si="4"/>
+        <v>235599.99999999997</v>
+      </c>
+      <c r="N28">
         <f t="shared" si="5"/>
-        <v>4.142670705571054E-3</v>
-      </c>
-      <c r="L28" s="9">
-        <f t="shared" si="2"/>
-        <v>383344</v>
-      </c>
-      <c r="M28" s="8">
-        <f>(E28-E27)*2*PI()/(D28-D27)</f>
-        <v>235599.99999999997</v>
-      </c>
-      <c r="N28">
-        <f t="shared" si="3"/>
         <v>122904.54858281543</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>26</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29">
         <v>1</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C29">
         <v>26</v>
       </c>
-      <c r="D29" s="6">
-        <f t="shared" si="4"/>
+      <c r="D29" s="5">
+        <f t="shared" si="6"/>
         <v>2.1495107629824903</v>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="6">
         <v>130000</v>
       </c>
-      <c r="F29" s="4">
+      <c r="F29" s="3">
         <v>3.6</v>
       </c>
       <c r="G29">
         <v>0.01</v>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="3">
         <v>0.49</v>
       </c>
       <c r="I29">
         <v>0.01</v>
       </c>
-      <c r="J29" s="5">
-        <f t="shared" si="0"/>
+      <c r="J29" s="4">
+        <f t="shared" si="1"/>
         <v>0.1361111111111111</v>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="4">
+        <f t="shared" si="7"/>
+        <v>3.1558641975308645E-3</v>
+      </c>
+      <c r="L29" s="8">
+        <f t="shared" si="3"/>
+        <v>379999.99999999994</v>
+      </c>
+      <c r="M29" s="7">
+        <f t="shared" si="4"/>
+        <v>296399.99999999919</v>
+      </c>
+      <c r="N29">
         <f t="shared" si="5"/>
-        <v>3.1558641975308645E-3</v>
-      </c>
-      <c r="L29" s="9">
-        <f t="shared" si="2"/>
-        <v>379999.99999999994</v>
-      </c>
-      <c r="M29" s="8">
-        <f>(E29-E28)*2*PI()/(D29-D28)</f>
-        <v>296399.99999999919</v>
-      </c>
-      <c r="N29">
-        <f t="shared" si="3"/>
         <v>125826.00176929946</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>27</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30">
         <v>0</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C30">
         <v>27</v>
       </c>
-      <c r="D30" s="6">
-        <f t="shared" si="4"/>
+      <c r="D30" s="5">
+        <f t="shared" si="6"/>
         <v>2.232184253866432</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="6">
         <v>132700</v>
       </c>
-      <c r="F30" s="4">
+      <c r="F30" s="3">
         <v>2.7</v>
       </c>
       <c r="G30">
         <v>0.01</v>
       </c>
-      <c r="H30" s="4">
+      <c r="H30" s="3">
         <v>0.39</v>
       </c>
       <c r="I30">
         <v>0.01</v>
       </c>
-      <c r="J30" s="5">
-        <f t="shared" si="0"/>
+      <c r="J30" s="4">
+        <f t="shared" si="1"/>
         <v>0.14444444444444443</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="4">
+        <f t="shared" si="7"/>
+        <v>4.2386831275720164E-3</v>
+      </c>
+      <c r="L30" s="8">
+        <f t="shared" si="3"/>
+        <v>373525.9259259259</v>
+      </c>
+      <c r="M30" s="7">
+        <f t="shared" si="4"/>
+        <v>205200.00000000055</v>
+      </c>
+      <c r="N30">
         <f t="shared" si="5"/>
-        <v>4.2386831275720164E-3</v>
-      </c>
-      <c r="L30" s="9">
-        <f t="shared" si="2"/>
-        <v>373525.9259259259</v>
-      </c>
-      <c r="M30" s="8">
-        <f>(E30-E29)*2*PI()/(D30-D29)</f>
-        <v>205200.00000000055</v>
-      </c>
-      <c r="N30">
-        <f t="shared" si="3"/>
         <v>128532.48334244174</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>28</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B31">
         <v>1</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31">
         <v>28</v>
       </c>
-      <c r="D31" s="6">
-        <f t="shared" si="4"/>
+      <c r="D31" s="5">
+        <f t="shared" si="6"/>
         <v>2.3148577447503738</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="6">
         <v>136000</v>
       </c>
-      <c r="F31" s="4">
+      <c r="F31" s="3">
         <v>3.91</v>
       </c>
       <c r="G31">
         <v>0.01</v>
       </c>
-      <c r="H31" s="4">
+      <c r="H31" s="3">
         <v>0.33</v>
       </c>
       <c r="I31">
         <v>0.01</v>
       </c>
-      <c r="J31" s="5">
-        <f t="shared" si="0"/>
+      <c r="J31" s="4">
+        <f t="shared" si="1"/>
         <v>8.4398976982097182E-2</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="4">
+        <f t="shared" si="7"/>
+        <v>2.7733989181127801E-3</v>
+      </c>
+      <c r="L31" s="8">
+        <f t="shared" si="3"/>
+        <v>369142.85714285716</v>
+      </c>
+      <c r="M31" s="7">
+        <f t="shared" si="4"/>
+        <v>250800.00000000067</v>
+      </c>
+      <c r="N31">
         <f t="shared" si="5"/>
-        <v>2.7733989181127801E-3</v>
-      </c>
-      <c r="L31" s="9">
-        <f t="shared" si="2"/>
-        <v>369142.85714285716</v>
-      </c>
-      <c r="M31" s="8">
-        <f>(E31-E30)*2*PI()/(D31-D30)</f>
-        <v>250800.00000000067</v>
-      </c>
-      <c r="N31">
-        <f t="shared" si="3"/>
         <v>131019.36932387472</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>29</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32">
         <v>0</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32">
         <v>29</v>
       </c>
-      <c r="D32" s="6">
-        <f t="shared" si="4"/>
+      <c r="D32" s="5">
+        <f t="shared" si="6"/>
         <v>2.3975312356343159</v>
       </c>
-      <c r="E32" s="7">
+      <c r="E32" s="6">
         <v>138700</v>
       </c>
-      <c r="F32" s="4">
+      <c r="F32" s="3">
         <v>4.16</v>
       </c>
       <c r="G32">
         <v>0.01</v>
       </c>
-      <c r="H32" s="4">
+      <c r="H32" s="3">
         <v>0.32</v>
       </c>
       <c r="I32">
         <v>0.01</v>
       </c>
-      <c r="J32" s="5">
-        <f t="shared" si="0"/>
+      <c r="J32" s="4">
+        <f t="shared" si="1"/>
         <v>7.6923076923076927E-2</v>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="4">
+        <f t="shared" si="7"/>
+        <v>2.5887573964497044E-3</v>
+      </c>
+      <c r="L32" s="8">
+        <f t="shared" si="3"/>
+        <v>363489.6551724138</v>
+      </c>
+      <c r="M32" s="7">
+        <f t="shared" si="4"/>
+        <v>205199.99999999945</v>
+      </c>
+      <c r="N32">
         <f t="shared" si="5"/>
-        <v>2.5887573964497044E-3</v>
-      </c>
-      <c r="L32" s="9">
-        <f t="shared" si="2"/>
-        <v>363489.6551724138</v>
-      </c>
-      <c r="M32" s="8">
-        <f>(E32-E31)*2*PI()/(D32-D31)</f>
-        <v>205199.99999999945</v>
-      </c>
-      <c r="N32">
-        <f t="shared" si="3"/>
         <v>133282.41091061567</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>30</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33">
         <v>1</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33">
         <v>30</v>
       </c>
-      <c r="D33" s="6">
-        <f t="shared" si="4"/>
+      <c r="D33" s="5">
+        <f t="shared" si="6"/>
         <v>2.4802047265182576</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="6">
         <v>141200</v>
       </c>
-      <c r="F33" s="4">
+      <c r="F33" s="3">
         <v>4.1100000000000003</v>
       </c>
       <c r="G33">
         <v>0.01</v>
       </c>
-      <c r="H33" s="4">
+      <c r="H33" s="3">
         <v>0.28000000000000003</v>
       </c>
       <c r="I33">
         <v>0.01</v>
       </c>
-      <c r="J33" s="5">
-        <f t="shared" si="0"/>
+      <c r="J33" s="4">
+        <f t="shared" si="1"/>
         <v>6.8126520681265207E-2</v>
       </c>
-      <c r="K33" s="5">
+      <c r="K33" s="4">
+        <f t="shared" si="7"/>
+        <v>2.5988479821928596E-3</v>
+      </c>
+      <c r="L33" s="8">
+        <f t="shared" si="3"/>
+        <v>357706.66666666669</v>
+      </c>
+      <c r="M33" s="7">
+        <f t="shared" si="4"/>
+        <v>190000.00000000049</v>
+      </c>
+      <c r="N33">
         <f t="shared" si="5"/>
-        <v>2.5988479821928596E-3</v>
-      </c>
-      <c r="L33" s="9">
-        <f t="shared" si="2"/>
-        <v>357706.66666666669</v>
-      </c>
-      <c r="M33" s="8">
-        <f>(E33-E32)*2*PI()/(D33-D32)</f>
-        <v>190000.00000000049</v>
-      </c>
-      <c r="N33">
-        <f t="shared" si="3"/>
         <v>135317.74173407519</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>31</v>
       </c>
-      <c r="B34" s="3">
+      <c r="B34">
         <v>0</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34">
         <v>31</v>
       </c>
-      <c r="D34" s="6">
-        <f t="shared" si="4"/>
+      <c r="D34" s="5">
+        <f t="shared" si="6"/>
         <v>2.5628782174021993</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="6">
         <v>143500</v>
       </c>
-      <c r="F34" s="4">
+      <c r="F34" s="3">
         <v>3.52</v>
       </c>
       <c r="G34">
         <v>0.01</v>
       </c>
-      <c r="H34" s="4">
+      <c r="H34" s="3">
         <v>0.2</v>
       </c>
       <c r="I34">
         <v>0.01</v>
       </c>
-      <c r="J34" s="5">
-        <f t="shared" si="0"/>
+      <c r="J34" s="4">
+        <f t="shared" si="1"/>
         <v>5.6818181818181823E-2</v>
       </c>
-      <c r="K34" s="5">
+      <c r="K34" s="4">
+        <f t="shared" si="7"/>
+        <v>3.0023243801652892E-3</v>
+      </c>
+      <c r="L34" s="8">
+        <f t="shared" si="3"/>
+        <v>351806.45161290327</v>
+      </c>
+      <c r="M34" s="7">
+        <f t="shared" si="4"/>
+        <v>174800.00000000044</v>
+      </c>
+      <c r="N34">
         <f t="shared" si="5"/>
-        <v>3.0023243801652892E-3</v>
-      </c>
-      <c r="L34" s="9">
-        <f t="shared" si="2"/>
-        <v>351806.45161290327</v>
-      </c>
-      <c r="M34" s="8">
-        <f>(E34-E33)*2*PI()/(D34-D33)</f>
-        <v>174800.00000000044</v>
-      </c>
-      <c r="N34">
-        <f t="shared" si="3"/>
         <v>137121.88446568334</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>32</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B35">
         <v>1</v>
       </c>
-      <c r="C35" s="3">
+      <c r="C35">
         <v>32</v>
       </c>
-      <c r="D35" s="6">
-        <f t="shared" si="4"/>
+      <c r="D35" s="5">
+        <f t="shared" si="6"/>
         <v>2.6455517082861415</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="6">
         <v>145300</v>
       </c>
-      <c r="F35" s="4">
+      <c r="F35" s="3">
         <v>3.59</v>
       </c>
       <c r="G35">
         <v>0.01</v>
       </c>
-      <c r="H35" s="4">
+      <c r="H35" s="3">
         <v>0.09</v>
       </c>
       <c r="I35">
         <v>0.01</v>
       </c>
-      <c r="J35" s="5">
-        <f t="shared" si="0"/>
+      <c r="J35" s="4">
+        <f t="shared" si="1"/>
         <v>2.5069637883008356E-2</v>
       </c>
-      <c r="K35" s="5">
+      <c r="K35" s="4">
+        <f t="shared" si="7"/>
+        <v>2.855347180732614E-3</v>
+      </c>
+      <c r="L35" s="8">
+        <f t="shared" si="3"/>
+        <v>345087.5</v>
+      </c>
+      <c r="M35" s="7">
+        <f t="shared" si="4"/>
+        <v>136799.99999999962</v>
+      </c>
+      <c r="N35">
         <f t="shared" si="5"/>
-        <v>2.855347180732614E-3</v>
-      </c>
-      <c r="L35" s="9">
-        <f t="shared" si="2"/>
-        <v>345087.5</v>
-      </c>
-      <c r="M35" s="8">
-        <f>(E35-E34)*2*PI()/(D35-D34)</f>
-        <v>136799.99999999962</v>
-      </c>
-      <c r="N35">
-        <f t="shared" si="3"/>
         <v>138691.75675784692</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="3"/>
-      <c r="D36" s="6"/>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D36" s="5"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="3"/>
-      <c r="D37" s="6"/>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D37" s="5"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="3"/>
-      <c r="D38" s="6"/>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="3"/>
-      <c r="D39" s="6"/>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="3"/>
-      <c r="D40" s="6"/>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D40" s="5"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="3"/>
-      <c r="D41" s="6"/>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D41" s="5"/>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="3"/>
-      <c r="D42" s="6"/>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D42" s="5"/>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="3"/>
-      <c r="D43" s="6"/>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D43" s="5"/>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="3"/>
-      <c r="D44" s="6"/>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D44" s="5"/>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="3"/>
-      <c r="D45" s="6"/>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D45" s="5"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="3"/>
-      <c r="D46" s="6"/>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D46" s="5"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="3"/>
-      <c r="D47" s="6"/>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D47" s="5"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="3"/>
-      <c r="D48" s="6"/>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="D48" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>